<commit_message>
docs(report5): rebuild and reconcile report counts and evidence
</commit_message>
<xml_diff>
--- a/docs/report5/deliverables/Report5_Test Report.xlsx
+++ b/docs/report5/deliverables/Report5_Test Report.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="9" r:id="R7f19a7a1a1304e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="Rd5a9245e058148af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Statistics" sheetId="5" r:id="R0af362897e3e49ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature 1" sheetId="3" r:id="R2f96bec74439494a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature 2" sheetId="8" r:id="Raa40918a97944519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Traceability" sheetId="10" r:id="R01dee72c1e784cb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Traceability" sheetId="11" r:id="Rf4960ddbd2ee481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mandatory Features" sheetId="12" r:id="R8369d79ab5494f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Workflows" sheetId="13" r:id="Rbdf4e5fd37884c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="14" r:id="R892a4f9b152b4d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NFR Results" sheetId="15" r:id="R5cecc2e9609c44ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="16" r:id="Rbe78a2ba9a4d4495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="9" r:id="Ref4137d12e964f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R3935e7c82cda4c6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Statistics" sheetId="5" r:id="R9eae920998ee4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature 1" sheetId="3" r:id="Rc8441777650041a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature 2" sheetId="8" r:id="R7afc504f5e3d4957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Traceability" sheetId="10" r:id="R82d529dcadbf4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Traceability" sheetId="11" r:id="Rb2a9be4ddba548f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mandatory Features" sheetId="12" r:id="R8daae115ea9b4898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Workflows" sheetId="13" r:id="Rf5b82248b57d44b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="14" r:id="R9abd5d8f87764b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NFR Results" sheetId="15" r:id="R61802114fac8416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="16" r:id="R268c81dbb6694123"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="ACTION">#REF!</x:definedName>
@@ -1688,7 +1688,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3965ab6e8d6c40f8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8abe0fe221544185"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2640,8 +2640,8 @@
     <x:mergeCell ref="B6:D6"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8351eb75ee454f05"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cdae0bdaeff4019"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbdb0da1b1d6421d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf31294fef6a54c91"/>
 </x:worksheet>
 </file>
 
@@ -5366,7 +5366,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62795814f8894d44"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cd51bcdaa3342c2"/>
 </x:worksheet>
 </file>
 
@@ -8753,7 +8753,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1107b30c04844fa"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refd7b65739de47a0"/>
 </x:worksheet>
 </file>
 

</xml_diff>